<commit_message>
Refactor lifetime gains essay: Clarify rules on Roth reform and estate tax, enhance readability, and remove redundant content.
</commit_message>
<xml_diff>
--- a/internal/analysis/calibration_comparison.xlsx
+++ b/internal/analysis/calibration_comparison.xlsx
@@ -166,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -186,11 +186,32 @@
       <top style="double"/>
       <bottom style="double"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -246,6 +267,7 @@
     <xf numFmtId="0" fontId="15" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -649,14 +671,14 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Moderate
-$2.5M–$10M</t>
+          <t>Moderate (Published)
+$2M–$6M</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Aggressive
-$1.25M–$5M</t>
+$1.25M–$4M</t>
         </is>
       </c>
     </row>
@@ -673,7 +695,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>$2.5M</t>
+          <t>$2M</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -695,7 +717,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>$5M</t>
+          <t>$4M</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -717,12 +739,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>$10M</t>
+          <t>$6M</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>$5M</t>
+          <t>$4M</t>
         </is>
       </c>
     </row>
@@ -739,12 +761,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>$7.5M</t>
+          <t>$4M</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>$3.75M</t>
+          <t>$2.75M</t>
         </is>
       </c>
     </row>
@@ -761,12 +783,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>~$17.5M</t>
+          <t>~$11.2M</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>~$8.75M</t>
+          <t>~$7.4M</t>
         </is>
       </c>
     </row>
@@ -778,17 +800,17 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>+$60-178B</t>
+          <t>+$30-150B</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>+$85-203B</t>
+          <t>+$45-170B</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>+$105-228B</t>
+          <t>+$70-200B</t>
         </is>
       </c>
     </row>
@@ -827,12 +849,12 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>$3.86M (saves $660K)</t>
+          <t>$5.55M (pays $1.03M more)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>$5.50M (pays $980K more)</t>
+          <t>$6.06M (pays $1.54M more)</t>
         </is>
       </c>
     </row>
@@ -849,12 +871,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>$33.3M (+$10.7M)</t>
+          <t>$33.7M (+$11.1M)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>$34.4M (+$11.8M)</t>
+          <t>$34.2M (+$11.6M)</t>
         </is>
       </c>
     </row>
@@ -962,7 +984,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Three sliding scale calibrations compared across case studies and revenue</t>
+          <t>Three sliding scale calibrations. Moderate = the PUBLISHED calibration ($2M/$6M).</t>
         </is>
       </c>
     </row>
@@ -984,19 +1006,19 @@
           <t>Generous</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n"/>
+      <c r="C5" s="41" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n"/>
+          <t>Moderate (Published)</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="n"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Aggressive</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n"/>
+      <c r="G5" s="41" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -1007,15 +1029,15 @@
       <c r="B6" s="13" t="n">
         <v>3000000</v>
       </c>
-      <c r="C6" s="14" t="n"/>
+      <c r="C6" s="41" t="n"/>
       <c r="D6" s="13" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="E6" s="14" t="n"/>
+        <v>2000000</v>
+      </c>
+      <c r="E6" s="41" t="n"/>
       <c r="F6" s="13" t="n">
         <v>1250000</v>
       </c>
-      <c r="G6" s="14" t="n"/>
+      <c r="G6" s="41" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -1026,15 +1048,15 @@
       <c r="B7" s="13" t="n">
         <v>25000000</v>
       </c>
-      <c r="C7" s="14" t="n"/>
+      <c r="C7" s="41" t="n"/>
       <c r="D7" s="13" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E7" s="14" t="n"/>
+        <v>6000000</v>
+      </c>
+      <c r="E7" s="41" t="n"/>
       <c r="F7" s="13" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="G7" s="14" t="n"/>
+        <v>4000000</v>
+      </c>
+      <c r="G7" s="41" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -1045,15 +1067,15 @@
       <c r="B8" s="13" t="n">
         <v>6000000</v>
       </c>
-      <c r="C8" s="14" t="n"/>
+      <c r="C8" s="41" t="n"/>
       <c r="D8" s="13" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="E8" s="14" t="n"/>
+        <v>4000000</v>
+      </c>
+      <c r="E8" s="41" t="n"/>
       <c r="F8" s="13" t="n">
         <v>2500000</v>
       </c>
-      <c r="G8" s="14" t="n"/>
+      <c r="G8" s="41" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -1064,15 +1086,15 @@
       <c r="B9" s="13" t="n">
         <v>50000000</v>
       </c>
-      <c r="C9" s="14" t="n"/>
+      <c r="C9" s="41" t="n"/>
       <c r="D9" s="13" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E9" s="14" t="n"/>
+        <v>12000000</v>
+      </c>
+      <c r="E9" s="41" t="n"/>
       <c r="F9" s="13" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="G9" s="14" t="n"/>
+        <v>8000000</v>
+      </c>
+      <c r="G9" s="41" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -1083,15 +1105,15 @@
       <c r="B10" s="13" t="n">
         <v>22000000</v>
       </c>
-      <c r="C10" s="14" t="n"/>
+      <c r="C10" s="41" t="n"/>
       <c r="D10" s="13" t="n">
-        <v>7500000</v>
-      </c>
-      <c r="E10" s="14" t="n"/>
+        <v>4000000</v>
+      </c>
+      <c r="E10" s="41" t="n"/>
       <c r="F10" s="13" t="n">
-        <v>3750000</v>
-      </c>
-      <c r="G10" s="14" t="n"/>
+        <v>2750000</v>
+      </c>
+      <c r="G10" s="41" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -1102,15 +1124,15 @@
       <c r="B11" s="13" t="n">
         <v>39242424</v>
       </c>
-      <c r="C11" s="14" t="n"/>
+      <c r="C11" s="41" t="n"/>
       <c r="D11" s="13" t="n">
-        <v>17518939</v>
-      </c>
-      <c r="E11" s="14" t="n"/>
+        <v>11212121</v>
+      </c>
+      <c r="E11" s="41" t="n"/>
       <c r="F11" s="13" t="n">
-        <v>8759470</v>
-      </c>
-      <c r="G11" s="14" t="n"/>
+        <v>7357955</v>
+      </c>
+      <c r="G11" s="41" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
@@ -1305,16 +1327,16 @@
         <v>0</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>2220</v>
+        <v>29600</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>0.0008</v>
+        <v>0.0106</v>
       </c>
       <c r="I5" s="19" t="n">
-        <v>118523</v>
+        <v>161623</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>0.0423</v>
+        <v>0.0577</v>
       </c>
     </row>
     <row r="6">
@@ -1339,16 +1361,16 @@
         <v>0.1133</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>4717500</v>
+        <v>5550000</v>
       </c>
       <c r="H6" s="18" t="n">
-        <v>0.2483</v>
+        <v>0.2921</v>
       </c>
       <c r="I6" s="20" t="n">
-        <v>5873750</v>
+        <v>6058750</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>0.3091</v>
+        <v>0.3189</v>
       </c>
     </row>
     <row r="7">
@@ -1373,16 +1395,16 @@
         <v>0.3155</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>32837500</v>
+        <v>33670000</v>
       </c>
       <c r="H7" s="18" t="n">
-        <v>0.3457</v>
+        <v>0.3544</v>
       </c>
       <c r="I7" s="20" t="n">
-        <v>33993750</v>
+        <v>34178750</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.3578</v>
+        <v>0.3598</v>
       </c>
     </row>
     <row r="8">
@@ -1407,16 +1429,16 @@
         <v>0.08069999999999999</v>
       </c>
       <c r="G8" s="20" t="n">
-        <v>3237500</v>
+        <v>4070000</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>0.2158</v>
+        <v>0.2713</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>4393750</v>
+        <v>4578750</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>0.2929</v>
+        <v>0.3053</v>
       </c>
     </row>
     <row r="9">
@@ -1543,11 +1565,11 @@
       </c>
       <c r="F14" s="14" t="n"/>
       <c r="G14" s="23" t="n">
-        <v>-552780</v>
+        <v>-525400</v>
       </c>
       <c r="H14" s="14" t="n"/>
       <c r="I14" s="23" t="n">
-        <v>-436477</v>
+        <v>-393377</v>
       </c>
       <c r="J14" s="14" t="n"/>
     </row>
@@ -1567,11 +1589,11 @@
       </c>
       <c r="F15" s="14" t="n"/>
       <c r="G15" s="24" t="n">
-        <v>197500</v>
+        <v>1030000</v>
       </c>
       <c r="H15" s="14" t="n"/>
       <c r="I15" s="24" t="n">
-        <v>1353750</v>
+        <v>1538750</v>
       </c>
       <c r="J15" s="14" t="n"/>
     </row>
@@ -1591,11 +1613,11 @@
       </c>
       <c r="F16" s="14" t="n"/>
       <c r="G16" s="24" t="n">
-        <v>10227500</v>
+        <v>11060000</v>
       </c>
       <c r="H16" s="14" t="n"/>
       <c r="I16" s="24" t="n">
-        <v>11383750</v>
+        <v>11568750</v>
       </c>
       <c r="J16" s="14" t="n"/>
     </row>
@@ -1615,11 +1637,11 @@
       </c>
       <c r="F17" s="14" t="n"/>
       <c r="G17" s="24" t="n">
-        <v>3237500</v>
+        <v>4070000</v>
       </c>
       <c r="H17" s="14" t="n"/>
       <c r="I17" s="24" t="n">
-        <v>4393750</v>
+        <v>4578750</v>
       </c>
       <c r="J17" s="14" t="n"/>
     </row>
@@ -1879,13 +1901,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="18" t="n">
-        <v>0.074</v>
+        <v>0.1009</v>
       </c>
       <c r="I7" s="17" t="n">
-        <v>27750</v>
+        <v>37841</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>0.0139</v>
+        <v>0.0189</v>
       </c>
     </row>
     <row r="8">
@@ -1902,22 +1924,22 @@
         <v>0</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>0</v>
+        <v>0.0462</v>
       </c>
       <c r="F8" s="28" t="n">
-        <v>0</v>
+        <v>11562</v>
       </c>
       <c r="G8" s="27" t="n">
-        <v>0</v>
+        <v>0.0046</v>
       </c>
       <c r="H8" s="27" t="n">
-        <v>0.1233</v>
+        <v>0.1682</v>
       </c>
       <c r="I8" s="28" t="n">
-        <v>77083</v>
+        <v>105114</v>
       </c>
       <c r="J8" s="27" t="n">
-        <v>0.0308</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="9">
@@ -1934,22 +1956,22 @@
         <v>0</v>
       </c>
       <c r="E9" s="27" t="n">
-        <v>0.0247</v>
+        <v>0.0925</v>
       </c>
       <c r="F9" s="28" t="n">
-        <v>6167</v>
+        <v>46250</v>
       </c>
       <c r="G9" s="27" t="n">
-        <v>0.0021</v>
+        <v>0.0154</v>
       </c>
       <c r="H9" s="27" t="n">
-        <v>0.1727</v>
+        <v>0.2355</v>
       </c>
       <c r="I9" s="28" t="n">
-        <v>151083</v>
+        <v>206023</v>
       </c>
       <c r="J9" s="27" t="n">
-        <v>0.0504</v>
+        <v>0.0687</v>
       </c>
     </row>
     <row r="10">
@@ -1966,22 +1988,22 @@
         <v>0.0067</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>0.1233</v>
+        <v>0.2775</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>154167</v>
+        <v>416250</v>
       </c>
       <c r="G10" s="18" t="n">
-        <v>0.0308</v>
+        <v>0.0833</v>
       </c>
       <c r="H10" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>693750</v>
+        <v>878750</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>0.1388</v>
+        <v>0.1757</v>
       </c>
     </row>
     <row r="11">
@@ -1998,22 +2020,22 @@
         <v>0.0263</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>0.2713</v>
+        <v>0.37</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>746167</v>
+        <v>1480000</v>
       </c>
       <c r="G11" s="18" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.185</v>
       </c>
       <c r="H11" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I11" s="17" t="n">
-        <v>1803750</v>
+        <v>1988750</v>
       </c>
       <c r="J11" s="18" t="n">
-        <v>0.2255</v>
+        <v>0.2486</v>
       </c>
     </row>
     <row r="12">
@@ -2033,19 +2055,19 @@
         <v>0.37</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>1387500</v>
+        <v>2220000</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>0.1388</v>
+        <v>0.222</v>
       </c>
       <c r="H12" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I12" s="17" t="n">
-        <v>2543750</v>
+        <v>2728750</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>0.2544</v>
+        <v>0.2729</v>
       </c>
     </row>
     <row r="13">
@@ -2065,19 +2087,19 @@
         <v>0.37</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>3237500</v>
+        <v>4070000</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>0.2158</v>
+        <v>0.2713</v>
       </c>
       <c r="H13" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I13" s="17" t="n">
-        <v>4393750</v>
+        <v>4578750</v>
       </c>
       <c r="J13" s="18" t="n">
-        <v>0.2929</v>
+        <v>0.3053</v>
       </c>
     </row>
     <row r="14">
@@ -2097,19 +2119,19 @@
         <v>0.37</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>5087500</v>
+        <v>5920000</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>0.2544</v>
+        <v>0.296</v>
       </c>
       <c r="H14" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I14" s="17" t="n">
-        <v>6243750</v>
+        <v>6428750</v>
       </c>
       <c r="J14" s="18" t="n">
-        <v>0.3122</v>
+        <v>0.3214</v>
       </c>
     </row>
     <row r="15">
@@ -2129,19 +2151,19 @@
         <v>0.37</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>6937500</v>
+        <v>7770000</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.2775</v>
+        <v>0.3108</v>
       </c>
       <c r="H15" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I15" s="17" t="n">
-        <v>8093750</v>
+        <v>8278750</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.3237</v>
+        <v>0.3311</v>
       </c>
     </row>
     <row r="16">
@@ -2161,19 +2183,19 @@
         <v>0.37</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>8787500</v>
+        <v>9620000</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>0.2929</v>
+        <v>0.3207</v>
       </c>
       <c r="H16" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I16" s="17" t="n">
-        <v>9943750</v>
+        <v>10128750</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>0.3315</v>
+        <v>0.3376</v>
       </c>
     </row>
     <row r="17">
@@ -2193,19 +2215,19 @@
         <v>0.37</v>
       </c>
       <c r="F17" s="17" t="n">
-        <v>16187500</v>
+        <v>17020000</v>
       </c>
       <c r="G17" s="18" t="n">
-        <v>0.3237</v>
+        <v>0.3404</v>
       </c>
       <c r="H17" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I17" s="17" t="n">
-        <v>17343750</v>
+        <v>17528750</v>
       </c>
       <c r="J17" s="18" t="n">
-        <v>0.3469</v>
+        <v>0.3506</v>
       </c>
     </row>
     <row r="18">
@@ -2225,19 +2247,19 @@
         <v>0.37</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>34687500</v>
+        <v>35520000</v>
       </c>
       <c r="G18" s="18" t="n">
-        <v>0.3469</v>
+        <v>0.3552</v>
       </c>
       <c r="H18" s="18" t="n">
         <v>0.37</v>
       </c>
       <c r="I18" s="17" t="n">
-        <v>35843750</v>
+        <v>36028750</v>
       </c>
       <c r="J18" s="18" t="n">
-        <v>0.3584</v>
+        <v>0.3603</v>
       </c>
     </row>
   </sheetData>
@@ -2282,7 +2304,7 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Directional estimates. Formal scoring by JCT/CBO needed for legislation.</t>
+          <t>Directional estimates. Moderate NET reconciled to published essay; component lines below predate recalibration and need rebuild.</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2864,7 @@
       </c>
       <c r="H21" s="36" t="inlineStr">
         <is>
-          <t>Breakeven ~$17.5M; gains above offset losses below</t>
+          <t>Breakeven ~$11.2M; more gains taxed above current rates</t>
         </is>
       </c>
       <c r="I21" s="35" t="inlineStr">
@@ -2858,7 +2880,7 @@
       </c>
       <c r="L21" s="36" t="inlineStr">
         <is>
-          <t>Breakeven ~$8.75M; most gains taxed above current rates</t>
+          <t>Breakeven ~$7.4M; most gains taxed above current rates</t>
         </is>
       </c>
     </row>
@@ -2908,17 +2930,17 @@
       </c>
       <c r="B24" s="39" t="inlineStr">
         <is>
-          <t>+$60B</t>
+          <t>+$30B</t>
         </is>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
-          <t>+$188B</t>
+          <t>+$150B</t>
         </is>
       </c>
       <c r="D24" s="40" t="inlineStr">
         <is>
-          <t>Range: +$60B to +$188B/yr</t>
+          <t>Directional. Range +$30B to +$150B/yr</t>
         </is>
       </c>
       <c r="E24" s="38" t="inlineStr">
@@ -2928,17 +2950,17 @@
       </c>
       <c r="F24" s="39" t="inlineStr">
         <is>
-          <t>+$85B</t>
+          <t>+$45B</t>
         </is>
       </c>
       <c r="G24" s="39" t="inlineStr">
         <is>
-          <t>+$218B</t>
+          <t>+$170B</t>
         </is>
       </c>
       <c r="H24" s="40" t="inlineStr">
         <is>
-          <t>Range: +$85B to +$218B/yr</t>
+          <t>PER PUBLISHED ESSAY: +$45B to +$170B/yr (mid ~$108B)</t>
         </is>
       </c>
       <c r="I24" s="38" t="inlineStr">
@@ -2948,17 +2970,17 @@
       </c>
       <c r="J24" s="39" t="inlineStr">
         <is>
-          <t>+$105B</t>
+          <t>+$70B</t>
         </is>
       </c>
       <c r="K24" s="39" t="inlineStr">
         <is>
-          <t>+$243B</t>
+          <t>+$200B</t>
         </is>
       </c>
       <c r="L24" s="40" t="inlineStr">
         <is>
-          <t>Range: +$105B to +$243B/yr</t>
+          <t>Directional. Range +$70B to +$200B/yr</t>
         </is>
       </c>
     </row>

</xml_diff>